<commit_message>
Actualizacion pedidos 14.10: Comercial y Fabricacion
</commit_message>
<xml_diff>
--- a/Gastos/2026-Forecast-Codiagro P&L.xlsx
+++ b/Gastos/2026-Forecast-Codiagro P&L.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroquimicacodiagro365-my.sharepoint.com/personal/oscar_ocampo_codiagro_com/Documents/Escritorio/Presupuesto 2026/Calsif Comerciales/Gastos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="8_{D7C7D22D-CC9C-4A22-ADAD-C3153CF08886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B44AA6C-1BE5-4D5B-91FD-80411F7C8796}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{D7C7D22D-CC9C-4A22-ADAD-C3153CF08886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86189455-F23E-4076-9388-8AB2B4892F25}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="804" activeTab="2" xr2:uid="{DA978C05-6AA7-4636-9B27-353885F16E02}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="804" xr2:uid="{DA978C05-6AA7-4636-9B27-353885F16E02}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="24" r:id="rId1"/>
@@ -36,9 +36,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId12"/>
-    <pivotCache cacheId="9" r:id="rId13"/>
-    <pivotCache cacheId="23" r:id="rId14"/>
+    <pivotCache cacheId="34" r:id="rId12"/>
+    <pivotCache cacheId="35" r:id="rId13"/>
+    <pivotCache cacheId="36" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1611,7 +1611,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
@@ -1624,6 +1624,7 @@
     <numFmt numFmtId="170" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="171" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="172" formatCode="#,##0.000;\(#,##0.000\);\-"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="43" x14ac:knownFonts="1">
     <font>
@@ -2481,7 +2482,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="74">
+  <cellStyleXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
@@ -2556,8 +2557,9 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="187">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3040,18 +3042,9 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="12" fillId="0" borderId="0" xfId="73" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -3103,8 +3096,13 @@
     <xf numFmtId="172" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="74">
+  <cellStyles count="75">
     <cellStyle name="20% - Énfasis1 2" xfId="35" xr:uid="{1185DB90-4849-424E-B2AB-58A2E7F5B16C}"/>
     <cellStyle name="20% - Énfasis2 2" xfId="39" xr:uid="{CB031776-CD72-4FFD-8E18-B0CE5BE23EC1}"/>
     <cellStyle name="20% - Énfasis3 2" xfId="43" xr:uid="{A67BE943-F1C9-487C-87B9-E0FD4EC5A0F5}"/>
@@ -3139,6 +3137,7 @@
     <cellStyle name="Euro" xfId="14" xr:uid="{DEF02B32-61E3-467E-9A66-32FFE2362EC6}"/>
     <cellStyle name="Incorrecto 2" xfId="23" xr:uid="{FCD35F9B-C378-4262-A1BC-473C25788F95}"/>
     <cellStyle name="Millares" xfId="61" builtinId="3"/>
+    <cellStyle name="Millares 10" xfId="74" xr:uid="{85B7A6F9-DAEF-4274-9018-E3513C451E46}"/>
     <cellStyle name="Millares 2" xfId="9" xr:uid="{3E2A6486-DE8B-49EB-87D3-C439AD296424}"/>
     <cellStyle name="Millares 2 2" xfId="13" xr:uid="{4ACFEA2F-A484-48A0-B363-4588FD0384FF}"/>
     <cellStyle name="Millares 2 2 2" xfId="68" xr:uid="{7BB455AC-ECF8-43A4-99FD-F3B15DB08262}"/>
@@ -3180,80 +3179,7 @@
     <cellStyle name="Título 4" xfId="19" xr:uid="{F80139BF-3F45-41CD-BF67-DFFAEF585870}"/>
     <cellStyle name="Total 2" xfId="33" xr:uid="{05B74CE7-C7F2-435C-8726-12D1C31FD517}"/>
   </cellStyles>
-  <dxfs count="26">
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -9171,7 +9097,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{20404466-1C8F-4694-BEC9-2336FD9092D9}" name="TablaDinámica1" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Detalle sin Ajustar">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{20404466-1C8F-4694-BEC9-2336FD9092D9}" name="TablaDinámica1" cacheId="36" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Detalle sin Ajustar">
   <location ref="B3:O16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
@@ -9325,7 +9251,7 @@
     <dataField name="Total 2026 " fld="21" baseField="5" baseItem="0"/>
   </dataFields>
   <formats count="13">
-    <format dxfId="25">
+    <format dxfId="12">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -9334,10 +9260,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="11">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="3">
@@ -9348,7 +9274,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="9">
       <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -9357,7 +9283,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="8">
       <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -9366,7 +9292,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="7">
       <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -9375,7 +9301,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="6">
       <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -9384,7 +9310,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="5">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4" selected="0">
@@ -9396,7 +9322,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="4">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="0" count="1">
@@ -9405,7 +9331,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -9417,7 +9343,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -9429,7 +9355,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="1">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -9449,7 +9375,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="0">
       <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
   </formats>
@@ -9466,7 +9392,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{574F8F0F-CABA-44C9-861D-B64737513C38}" name="TablaDinámica13" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{574F8F0F-CABA-44C9-861D-B64737513C38}" name="TablaDinámica13" cacheId="35" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="P3:Q12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="12">
     <pivotField numFmtId="14" showAll="0"/>
@@ -9563,7 +9489,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BCFB44B8-C86C-4350-A9CC-CF0A10A66821}" name="TablaDinámica2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BCFB44B8-C86C-4350-A9CC-CF0A10A66821}" name="TablaDinámica2" cacheId="34" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A29:N33" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField numFmtId="14" showAll="0"/>
@@ -10277,10 +10203,10 @@
       </c>
       <c r="X6" s="77"/>
       <c r="Y6" s="78"/>
-      <c r="Z6" s="167" t="s">
+      <c r="Z6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="AA6" s="167"/>
+      <c r="AA6" s="183"/>
       <c r="AC6" s="74"/>
       <c r="AD6" s="75"/>
       <c r="AE6" s="75"/>
@@ -10289,10 +10215,10 @@
       </c>
       <c r="AG6" s="77"/>
       <c r="AH6" s="78"/>
-      <c r="AI6" s="167" t="s">
+      <c r="AI6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="AJ6" s="167"/>
+      <c r="AJ6" s="183"/>
       <c r="AL6" s="74"/>
       <c r="AM6" s="75"/>
       <c r="AN6" s="75"/>
@@ -10301,10 +10227,10 @@
       </c>
       <c r="AP6" s="77"/>
       <c r="AQ6" s="78"/>
-      <c r="AR6" s="167" t="s">
+      <c r="AR6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="AS6" s="167"/>
+      <c r="AS6" s="183"/>
       <c r="AU6" s="74"/>
       <c r="AV6" s="75"/>
       <c r="AW6" s="75"/>
@@ -10313,10 +10239,10 @@
       </c>
       <c r="AY6" s="77"/>
       <c r="AZ6" s="78"/>
-      <c r="BA6" s="167" t="s">
+      <c r="BA6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="BB6" s="167"/>
+      <c r="BB6" s="183"/>
       <c r="BD6" s="74"/>
       <c r="BE6" s="75"/>
       <c r="BF6" s="75"/>
@@ -10325,10 +10251,10 @@
       </c>
       <c r="BH6" s="77"/>
       <c r="BI6" s="78"/>
-      <c r="BJ6" s="167" t="s">
+      <c r="BJ6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="BK6" s="167"/>
+      <c r="BK6" s="183"/>
       <c r="BM6" s="74"/>
       <c r="BN6" s="75"/>
       <c r="BO6" s="75"/>
@@ -10337,10 +10263,10 @@
       </c>
       <c r="BQ6" s="77"/>
       <c r="BR6" s="78"/>
-      <c r="BS6" s="167" t="s">
+      <c r="BS6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="BT6" s="167"/>
+      <c r="BT6" s="183"/>
       <c r="BV6" s="74"/>
       <c r="BW6" s="75"/>
       <c r="BX6" s="75"/>
@@ -10349,10 +10275,10 @@
       </c>
       <c r="BZ6" s="77"/>
       <c r="CA6" s="78"/>
-      <c r="CB6" s="167" t="s">
+      <c r="CB6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="CC6" s="167"/>
+      <c r="CC6" s="183"/>
       <c r="CD6" s="103"/>
       <c r="CE6" s="74"/>
       <c r="CF6" s="75"/>
@@ -10362,10 +10288,10 @@
       </c>
       <c r="CI6" s="77"/>
       <c r="CJ6" s="78"/>
-      <c r="CK6" s="167" t="s">
+      <c r="CK6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="CL6" s="167"/>
+      <c r="CL6" s="183"/>
       <c r="CN6" s="74"/>
       <c r="CO6" s="75"/>
       <c r="CP6" s="75"/>
@@ -10374,10 +10300,10 @@
       </c>
       <c r="CR6" s="77"/>
       <c r="CS6" s="78"/>
-      <c r="CT6" s="167" t="s">
+      <c r="CT6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="CU6" s="167"/>
+      <c r="CU6" s="183"/>
       <c r="CW6" s="74"/>
       <c r="CX6" s="75"/>
       <c r="CY6" s="75"/>
@@ -10386,10 +10312,10 @@
       </c>
       <c r="DA6" s="77"/>
       <c r="DB6" s="78"/>
-      <c r="DC6" s="167" t="s">
+      <c r="DC6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="DD6" s="167"/>
+      <c r="DD6" s="183"/>
       <c r="DF6" s="74"/>
       <c r="DG6" s="75"/>
       <c r="DH6" s="75"/>
@@ -10398,10 +10324,10 @@
       </c>
       <c r="DJ6" s="77"/>
       <c r="DK6" s="78"/>
-      <c r="DL6" s="167" t="s">
+      <c r="DL6" s="183" t="s">
         <v>21</v>
       </c>
-      <c r="DM6" s="167"/>
+      <c r="DM6" s="183"/>
     </row>
     <row r="7" spans="2:117" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="79" t="s">
@@ -10416,7 +10342,7 @@
       <c r="E7" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="173" t="s">
+      <c r="F7" s="169" t="s">
         <v>22</v>
       </c>
       <c r="G7" s="80" t="s">
@@ -10440,7 +10366,7 @@
       <c r="N7" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="O7" s="173" t="s">
+      <c r="O7" s="169" t="s">
         <v>22</v>
       </c>
       <c r="P7" s="80" t="s">
@@ -10731,7 +10657,7 @@
       <c r="E8" s="110">
         <v>361.52999</v>
       </c>
-      <c r="F8" s="174">
+      <c r="F8" s="170">
         <v>0.58096972725484897</v>
       </c>
       <c r="G8" s="118">
@@ -10740,7 +10666,7 @@
       <c r="H8" s="110">
         <v>178.12350188020241</v>
       </c>
-      <c r="I8" s="174">
+      <c r="I8" s="170">
         <v>0.22108093655386021</v>
       </c>
       <c r="K8" s="82" t="s">
@@ -10755,7 +10681,7 @@
       <c r="N8" s="110">
         <v>407.98705999999993</v>
       </c>
-      <c r="O8" s="174">
+      <c r="O8" s="170">
         <v>0.3840091124487664</v>
       </c>
       <c r="P8" s="118">
@@ -10764,7 +10690,7 @@
       <c r="Q8" s="110">
         <v>-42.81983298277396</v>
       </c>
-      <c r="R8" s="174">
+      <c r="R8" s="170">
         <v>-2.8296639720854926E-2</v>
       </c>
       <c r="T8" s="82" t="s">
@@ -11090,7 +11016,7 @@
       <c r="H9" s="112">
         <v>-225.96264397487369</v>
       </c>
-      <c r="I9" s="175">
+      <c r="I9" s="171">
         <v>0.8166254818962938</v>
       </c>
       <c r="K9" s="74" t="s">
@@ -11114,7 +11040,7 @@
       <c r="Q9" s="112">
         <v>163.46424983383275</v>
       </c>
-      <c r="R9" s="175">
+      <c r="R9" s="171">
         <v>-0.31453493629370405</v>
       </c>
       <c r="T9" s="74" t="s">
@@ -11431,7 +11357,7 @@
       <c r="E10" s="115">
         <v>376.95908999999989</v>
       </c>
-      <c r="F10" s="176">
+      <c r="F10" s="172">
         <v>3.6179103695477419</v>
       </c>
       <c r="G10" s="115">
@@ -11455,7 +11381,7 @@
       <c r="N10" s="115">
         <v>503.26486</v>
       </c>
-      <c r="O10" s="176">
+      <c r="O10" s="172">
         <v>0.82377366965790111</v>
       </c>
       <c r="P10" s="115">
@@ -11779,7 +11705,7 @@
         <v>0.16743474724545993</v>
       </c>
       <c r="E11" s="87"/>
-      <c r="F11" s="177"/>
+      <c r="F11" s="173"/>
       <c r="G11" s="117">
         <v>0.65656560214972481</v>
       </c>
@@ -11795,7 +11721,7 @@
         <v>0.57502118070376973</v>
       </c>
       <c r="N11" s="87"/>
-      <c r="O11" s="177"/>
+      <c r="O11" s="173"/>
       <c r="P11" s="117">
         <v>0.65656560214972459</v>
       </c>
@@ -11999,7 +11925,7 @@
       <c r="C12" s="90"/>
       <c r="D12" s="91"/>
       <c r="E12" s="92"/>
-      <c r="F12" s="178"/>
+      <c r="F12" s="174"/>
       <c r="G12" s="93"/>
       <c r="H12" s="92"/>
       <c r="I12" s="94"/>
@@ -12007,7 +11933,7 @@
       <c r="L12" s="90"/>
       <c r="M12" s="91"/>
       <c r="N12" s="92"/>
-      <c r="O12" s="178"/>
+      <c r="O12" s="174"/>
       <c r="P12" s="93"/>
       <c r="Q12" s="92"/>
       <c r="R12" s="94"/>
@@ -12123,7 +12049,7 @@
       <c r="H13" s="120">
         <v>26.898993496442941</v>
       </c>
-      <c r="I13" s="179">
+      <c r="I13" s="175">
         <v>-0.19431336056979551</v>
       </c>
       <c r="K13" s="95" t="s">
@@ -12147,7 +12073,7 @@
       <c r="Q13" s="120">
         <v>9.8748134964428971</v>
       </c>
-      <c r="R13" s="179">
+      <c r="R13" s="175">
         <v>-6.4624891194072998E-2</v>
       </c>
       <c r="T13" s="95" t="s">
@@ -12462,7 +12388,7 @@
         <v>2.7957696506471303E-2</v>
       </c>
       <c r="E14" s="97"/>
-      <c r="F14" s="180"/>
+      <c r="F14" s="176"/>
       <c r="G14" s="101">
         <v>-0.17181593432666417</v>
       </c>
@@ -12478,7 +12404,7 @@
         <v>-0.15991689478049079</v>
       </c>
       <c r="N14" s="97"/>
-      <c r="O14" s="180"/>
+      <c r="O14" s="176"/>
       <c r="P14" s="101">
         <v>-0.1009761884468227</v>
       </c>
@@ -12682,7 +12608,7 @@
       <c r="C15" s="98"/>
       <c r="D15" s="98"/>
       <c r="E15" s="83"/>
-      <c r="F15" s="180"/>
+      <c r="F15" s="176"/>
       <c r="G15" s="83"/>
       <c r="H15" s="83"/>
       <c r="I15" s="84"/>
@@ -12690,7 +12616,7 @@
       <c r="L15" s="98"/>
       <c r="M15" s="98"/>
       <c r="N15" s="83"/>
-      <c r="O15" s="180"/>
+      <c r="O15" s="176"/>
       <c r="P15" s="83"/>
       <c r="Q15" s="83"/>
       <c r="R15" s="84"/>
@@ -12806,7 +12732,7 @@
       <c r="H16" s="112">
         <v>0</v>
       </c>
-      <c r="I16" s="175" t="s">
+      <c r="I16" s="171" t="s">
         <v>62</v>
       </c>
       <c r="K16" s="74" t="s">
@@ -12830,7 +12756,7 @@
       <c r="Q16" s="112">
         <v>0</v>
       </c>
-      <c r="R16" s="175" t="s">
+      <c r="R16" s="171" t="s">
         <v>62</v>
       </c>
       <c r="T16" s="74" t="s">
@@ -13156,7 +13082,7 @@
       <c r="H17" s="111">
         <v>79.883569163333291</v>
       </c>
-      <c r="I17" s="181">
+      <c r="I17" s="177">
         <v>-0.43572381563274742</v>
       </c>
       <c r="K17" s="74" t="s">
@@ -13180,7 +13106,7 @@
       <c r="Q17" s="111">
         <v>71.356439163333349</v>
       </c>
-      <c r="R17" s="181">
+      <c r="R17" s="177">
         <v>-0.53308631744594759</v>
       </c>
       <c r="T17" s="74" t="s">
@@ -13210,7 +13136,7 @@
       <c r="AC17" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="AD17" s="186">
+      <c r="AD17" s="182">
         <v>-107.70665</v>
       </c>
       <c r="AE17" s="3">
@@ -13506,7 +13432,7 @@
       <c r="H18" s="7">
         <v>79.883569163333291</v>
       </c>
-      <c r="I18" s="182">
+      <c r="I18" s="178">
         <v>-0.43572381563274742</v>
       </c>
       <c r="K18" s="99" t="s">
@@ -13530,7 +13456,7 @@
       <c r="Q18" s="7">
         <v>71.356439163333349</v>
       </c>
-      <c r="R18" s="182">
+      <c r="R18" s="178">
         <v>-0.53308631744594759</v>
       </c>
       <c r="T18" s="99" t="s">
@@ -13845,7 +13771,7 @@
         <v>-0.13345231591962509</v>
       </c>
       <c r="E19" s="83"/>
-      <c r="F19" s="180"/>
+      <c r="F19" s="176"/>
       <c r="G19" s="101">
         <v>-0.22754968236645082</v>
       </c>
@@ -13861,7 +13787,7 @@
         <v>-7.0225427745833902E-2</v>
       </c>
       <c r="N19" s="83"/>
-      <c r="O19" s="180"/>
+      <c r="O19" s="176"/>
       <c r="P19" s="101">
         <v>-8.8455640231213245E-2</v>
       </c>
@@ -14073,7 +13999,7 @@
       <c r="E20" s="124">
         <v>-149.33582500000006</v>
       </c>
-      <c r="F20" s="183">
+      <c r="F20" s="179">
         <v>2.2747981677111166</v>
       </c>
       <c r="G20" s="24">
@@ -14082,7 +14008,7 @@
       <c r="H20" s="24">
         <v>106.78256265977626</v>
       </c>
-      <c r="I20" s="184">
+      <c r="I20" s="180">
         <v>-0.3318636905766153</v>
       </c>
       <c r="K20" s="100" t="s">
@@ -14097,7 +14023,7 @@
       <c r="N20" s="124">
         <v>39.086579999999969</v>
       </c>
-      <c r="O20" s="183">
+      <c r="O20" s="179">
         <v>-0.15985503572698434</v>
       </c>
       <c r="P20" s="24">
@@ -14106,7 +14032,7 @@
       <c r="Q20" s="24">
         <v>81.23125265977626</v>
       </c>
-      <c r="R20" s="184">
+      <c r="R20" s="180">
         <v>-0.28337406165774537</v>
       </c>
       <c r="T20" s="100" t="s">
@@ -14421,7 +14347,7 @@
         <v>-0.10549461941315379</v>
       </c>
       <c r="E21" s="83"/>
-      <c r="F21" s="180"/>
+      <c r="F21" s="176"/>
       <c r="G21" s="101">
         <v>-0.39936561669311504</v>
       </c>
@@ -14437,7 +14363,7 @@
         <v>-0.23014232252632472</v>
       </c>
       <c r="N21" s="83"/>
-      <c r="O21" s="180"/>
+      <c r="O21" s="176"/>
       <c r="P21" s="101">
         <v>-0.18943182867803593</v>
       </c>
@@ -14649,7 +14575,7 @@
       <c r="E22" s="110">
         <v>227.62326499999983</v>
       </c>
-      <c r="F22" s="174">
+      <c r="F22" s="170">
         <v>5.905459903599815</v>
       </c>
       <c r="G22" s="110">
@@ -14673,7 +14599,7 @@
       <c r="N22" s="110">
         <v>542.35144000000003</v>
       </c>
-      <c r="O22" s="174">
+      <c r="O22" s="170">
         <v>1.4801623968682154</v>
       </c>
       <c r="P22" s="110">
@@ -14997,7 +14923,7 @@
         <v>6.1940127832306131E-2</v>
       </c>
       <c r="E23" s="88"/>
-      <c r="F23" s="185"/>
+      <c r="F23" s="181"/>
       <c r="G23" s="101">
         <v>0.25719998545660977</v>
       </c>
@@ -15013,7 +14939,7 @@
         <v>0.34487885817744501</v>
       </c>
       <c r="N23" s="88"/>
-      <c r="O23" s="185"/>
+      <c r="O23" s="181"/>
       <c r="P23" s="101">
         <v>0.46713377347168872</v>
       </c>
@@ -15244,7 +15170,7 @@
       <c r="C24" s="91"/>
       <c r="D24" s="91"/>
       <c r="E24" s="92"/>
-      <c r="F24" s="178"/>
+      <c r="F24" s="174"/>
       <c r="G24" s="93"/>
       <c r="H24" s="92"/>
       <c r="I24" s="94"/>
@@ -15252,7 +15178,7 @@
       <c r="L24" s="91"/>
       <c r="M24" s="91"/>
       <c r="N24" s="92"/>
-      <c r="O24" s="178"/>
+      <c r="O24" s="174"/>
       <c r="P24" s="93"/>
       <c r="Q24" s="92"/>
       <c r="R24" s="94"/>
@@ -15368,7 +15294,7 @@
       <c r="H25" s="112">
         <v>1.7004629999999992</v>
       </c>
-      <c r="I25" s="175">
+      <c r="I25" s="171">
         <v>-8.1622225305955573E-2</v>
       </c>
       <c r="K25" s="74" t="s">
@@ -15392,7 +15318,7 @@
       <c r="Q25" s="112">
         <v>1.7004629999999992</v>
       </c>
-      <c r="R25" s="175">
+      <c r="R25" s="171">
         <v>-8.1622225305955573E-2</v>
       </c>
       <c r="T25" s="74" t="s">
@@ -15718,7 +15644,7 @@
       <c r="H26" s="112">
         <v>3.0652699999999999</v>
       </c>
-      <c r="I26" s="175" t="s">
+      <c r="I26" s="171" t="s">
         <v>62</v>
       </c>
       <c r="K26" s="74" t="s">
@@ -15742,7 +15668,7 @@
       <c r="Q26" s="112">
         <v>2.0000000000000002E-5</v>
       </c>
-      <c r="R26" s="175" t="s">
+      <c r="R26" s="171" t="s">
         <v>62</v>
       </c>
       <c r="T26" s="74" t="s">
@@ -16054,7 +15980,7 @@
       <c r="E27" s="110">
         <v>210.63419499999986</v>
       </c>
-      <c r="F27" s="174">
+      <c r="F27" s="170">
         <v>5.3371032013239459</v>
       </c>
       <c r="G27" s="110">
@@ -16078,7 +16004,7 @@
       <c r="N27" s="110">
         <v>523.18675999999994</v>
       </c>
-      <c r="O27" s="174">
+      <c r="O27" s="170">
         <v>1.4277349443423064</v>
       </c>
       <c r="P27" s="110">
@@ -16402,7 +16328,7 @@
         <v>6.3420907267985938E-2</v>
       </c>
       <c r="E28" s="89"/>
-      <c r="F28" s="185"/>
+      <c r="F28" s="181"/>
       <c r="G28" s="126">
         <v>0.23134234891476743</v>
       </c>
@@ -16418,7 +16344,7 @@
         <v>0.34490881748558883</v>
       </c>
       <c r="N28" s="89"/>
-      <c r="O28" s="185"/>
+      <c r="O28" s="181"/>
       <c r="P28" s="126">
         <v>0.453366477407672</v>
       </c>
@@ -16634,7 +16560,7 @@
     </row>
     <row r="32" spans="2:117" x14ac:dyDescent="0.35">
       <c r="BM32" s="74"/>
-      <c r="BN32" s="172"/>
+      <c r="BN32" s="168"/>
       <c r="BO32" s="75"/>
       <c r="BP32" s="76" t="s">
         <v>21</v>
@@ -16646,7 +16572,7 @@
       </c>
       <c r="BT32" s="76"/>
     </row>
-    <row r="33" spans="65:72" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="65:101" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="BM33" s="79" t="s">
         <v>18</v>
       </c>
@@ -16672,7 +16598,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="34" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM34" s="82" t="s">
         <v>1</v>
       </c>
@@ -16697,8 +16623,11 @@
       <c r="BT34" s="125">
         <v>-8.1018252585747463E-2</v>
       </c>
-    </row>
-    <row r="35" spans="65:72" x14ac:dyDescent="0.35">
+      <c r="BW34" s="184">
+        <v>-3.6197427654381727E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM35" s="74" t="s">
         <v>2</v>
       </c>
@@ -16724,7 +16653,7 @@
         <v>-8.2181667792948221E-2</v>
       </c>
     </row>
-    <row r="36" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="36" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM36" s="85" t="s">
         <v>3</v>
       </c>
@@ -16749,8 +16678,12 @@
       <c r="BT36" s="116">
         <v>-8.040969679204335E-2</v>
       </c>
-    </row>
-    <row r="37" spans="65:72" x14ac:dyDescent="0.35">
+      <c r="CW36" s="69">
+        <f>CX8*BW34</f>
+        <v>-41.352208489381781</v>
+      </c>
+    </row>
+    <row r="37" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM37" s="86" t="s">
         <v>4</v>
       </c>
@@ -16767,8 +16700,12 @@
       </c>
       <c r="BS37" s="88"/>
       <c r="BT37" s="128"/>
-    </row>
-    <row r="38" spans="65:72" x14ac:dyDescent="0.35">
+      <c r="CN37" s="69">
+        <f>BW34*CO8</f>
+        <v>-44.35349648488824</v>
+      </c>
+    </row>
+    <row r="38" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM38" s="86"/>
       <c r="BN38" s="90"/>
       <c r="BO38" s="91"/>
@@ -16777,8 +16714,16 @@
       <c r="BR38" s="93"/>
       <c r="BS38" s="92"/>
       <c r="BT38" s="129"/>
-    </row>
-    <row r="39" spans="65:72" x14ac:dyDescent="0.35">
+      <c r="BW38" s="70">
+        <f>BW34*625</f>
+        <v>-22.623392283988579</v>
+      </c>
+      <c r="CE38" s="69">
+        <f>BW34*CF8</f>
+        <v>-33.014045241291406</v>
+      </c>
+    </row>
+    <row r="39" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM39" s="95" t="s">
         <v>5</v>
       </c>
@@ -16804,7 +16749,7 @@
         <v>-0.2477832710433614</v>
       </c>
     </row>
-    <row r="40" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="40" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM40" s="96" t="s">
         <v>6</v>
       </c>
@@ -16822,7 +16767,7 @@
       <c r="BS40" s="97"/>
       <c r="BT40" s="113"/>
     </row>
-    <row r="41" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="41" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM41" s="96"/>
       <c r="BN41" s="98"/>
       <c r="BO41" s="98"/>
@@ -16832,7 +16777,7 @@
       <c r="BS41" s="83"/>
       <c r="BT41" s="113"/>
     </row>
-    <row r="42" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="42" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM42" s="74" t="s">
         <v>7</v>
       </c>
@@ -16858,7 +16803,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="43" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM43" s="74" t="s">
         <v>8</v>
       </c>
@@ -16884,7 +16829,7 @@
         <v>-0.14262306387477719</v>
       </c>
     </row>
-    <row r="44" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="44" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM44" s="99" t="s">
         <v>9</v>
       </c>
@@ -16910,7 +16855,7 @@
         <v>-0.20542224655366437</v>
       </c>
     </row>
-    <row r="45" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="45" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM45" s="74" t="s">
         <v>6</v>
       </c>
@@ -16928,7 +16873,7 @@
       <c r="BS45" s="83"/>
       <c r="BT45" s="113"/>
     </row>
-    <row r="46" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="46" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM46" s="100" t="s">
         <v>10</v>
       </c>
@@ -16954,7 +16899,7 @@
         <v>-0.22942451931680696</v>
       </c>
     </row>
-    <row r="47" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="47" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM47" s="74" t="s">
         <v>6</v>
       </c>
@@ -16972,7 +16917,7 @@
       <c r="BS47" s="83"/>
       <c r="BT47" s="113"/>
     </row>
-    <row r="48" spans="65:72" x14ac:dyDescent="0.35">
+    <row r="48" spans="65:101" x14ac:dyDescent="0.35">
       <c r="BM48" s="82" t="s">
         <v>11</v>
       </c>
@@ -17126,17 +17071,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="CB6:CC6"/>
+    <mergeCell ref="CK6:CL6"/>
+    <mergeCell ref="CT6:CU6"/>
+    <mergeCell ref="DC6:DD6"/>
+    <mergeCell ref="DL6:DM6"/>
     <mergeCell ref="BS6:BT6"/>
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="AI6:AJ6"/>
     <mergeCell ref="AR6:AS6"/>
     <mergeCell ref="BA6:BB6"/>
     <mergeCell ref="BJ6:BK6"/>
-    <mergeCell ref="CB6:CC6"/>
-    <mergeCell ref="CK6:CL6"/>
-    <mergeCell ref="CT6:CU6"/>
-    <mergeCell ref="DC6:DD6"/>
-    <mergeCell ref="DL6:DM6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="15" orientation="landscape" r:id="rId1"/>
@@ -19249,16 +19194,16 @@
       <c r="B3" s="162" t="s">
         <v>427</v>
       </c>
-      <c r="C3" s="169" t="s">
+      <c r="C3" s="167" t="s">
         <v>314</v>
       </c>
-      <c r="D3" s="169" t="s">
+      <c r="D3" s="167" t="s">
         <v>315</v>
       </c>
-      <c r="E3" s="169" t="s">
+      <c r="E3" s="167" t="s">
         <v>316</v>
       </c>
-      <c r="F3" s="170" t="s">
+      <c r="F3" s="26" t="s">
         <v>317</v>
       </c>
       <c r="G3" t="s">
@@ -19293,16 +19238,16 @@
       <c r="B4" s="67" t="s">
         <v>78</v>
       </c>
-      <c r="C4" s="168">
+      <c r="C4" s="19">
         <v>983817.13</v>
       </c>
-      <c r="D4" s="168">
+      <c r="D4" s="19">
         <v>1470428.15</v>
       </c>
-      <c r="E4" s="168">
+      <c r="E4" s="19">
         <v>1533789.4100000004</v>
       </c>
-      <c r="F4" s="168">
+      <c r="F4" s="19">
         <v>1462146.28</v>
       </c>
       <c r="G4" s="19">
@@ -19337,16 +19282,16 @@
       <c r="B5" s="67" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="168">
+      <c r="C5" s="19">
         <v>-84878.079999999987</v>
       </c>
-      <c r="D5" s="168">
+      <c r="D5" s="19">
         <v>50005.570000000007</v>
       </c>
-      <c r="E5" s="168">
+      <c r="E5" s="19">
         <v>83552.76999999999</v>
       </c>
-      <c r="F5" s="168">
+      <c r="F5" s="19">
         <v>8645.1999999999989</v>
       </c>
       <c r="G5" s="19">
@@ -19373,7 +19318,7 @@
       <c r="N5" s="19">
         <v>0</v>
       </c>
-      <c r="O5" s="171">
+      <c r="O5" s="19">
         <v>-62628.5</v>
       </c>
     </row>
@@ -19381,16 +19326,16 @@
       <c r="B6" s="67" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="168">
+      <c r="C6" s="19">
         <v>-417787.47</v>
       </c>
-      <c r="D6" s="168">
+      <c r="D6" s="19">
         <v>-406242.7300000001</v>
       </c>
-      <c r="E6" s="168">
+      <c r="E6" s="19">
         <v>-469252.69999999995</v>
       </c>
-      <c r="F6" s="168">
+      <c r="F6" s="19">
         <v>-514848.29</v>
       </c>
       <c r="G6" s="19">
@@ -19417,7 +19362,7 @@
       <c r="N6" s="19">
         <v>-449145.32999999996</v>
       </c>
-      <c r="O6" s="171">
+      <c r="O6" s="19">
         <v>-5170904.3499999996</v>
       </c>
     </row>
@@ -19425,16 +19370,16 @@
       <c r="B7" s="67" t="s">
         <v>119</v>
       </c>
-      <c r="C7" s="168">
+      <c r="C7" s="19">
         <v>-111532.01</v>
       </c>
-      <c r="D7" s="168">
+      <c r="D7" s="19">
         <v>-142927.20000000001</v>
       </c>
-      <c r="E7" s="168">
+      <c r="E7" s="19">
         <v>-146233.31</v>
       </c>
-      <c r="F7" s="168">
+      <c r="F7" s="19">
         <v>-130047.67000000001</v>
       </c>
       <c r="G7" s="19">
@@ -19461,7 +19406,7 @@
       <c r="N7" s="19">
         <v>-431632.79</v>
       </c>
-      <c r="O7" s="171">
+      <c r="O7" s="19">
         <v>-2006502.5899999999</v>
       </c>
     </row>
@@ -19469,16 +19414,16 @@
       <c r="B8" s="67" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="168">
-        <v>0</v>
-      </c>
-      <c r="D8" s="168">
-        <v>0</v>
-      </c>
-      <c r="E8" s="168">
-        <v>0</v>
-      </c>
-      <c r="F8" s="168">
+      <c r="C8" s="19">
+        <v>0</v>
+      </c>
+      <c r="D8" s="19">
+        <v>0</v>
+      </c>
+      <c r="E8" s="19">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19">
         <v>750.75</v>
       </c>
       <c r="G8" s="19">
@@ -19505,7 +19450,7 @@
       <c r="N8" s="19">
         <v>27150</v>
       </c>
-      <c r="O8" s="171">
+      <c r="O8" s="19">
         <v>168561.34</v>
       </c>
     </row>
@@ -19513,16 +19458,16 @@
       <c r="B9" s="67" t="s">
         <v>140</v>
       </c>
-      <c r="C9" s="168">
+      <c r="C9" s="19">
         <v>-103451.75999999995</v>
       </c>
-      <c r="D9" s="168">
+      <c r="D9" s="19">
         <v>-62498.880000000019</v>
       </c>
-      <c r="E9" s="168">
+      <c r="E9" s="19">
         <v>-110606.27000000002</v>
       </c>
-      <c r="F9" s="168">
+      <c r="F9" s="19">
         <v>-107706.65</v>
       </c>
       <c r="G9" s="19">
@@ -19549,7 +19494,7 @@
       <c r="N9" s="19">
         <v>-277596.2900000001</v>
       </c>
-      <c r="O9" s="171">
+      <c r="O9" s="19">
         <v>-1684026.025250294</v>
       </c>
     </row>
@@ -19557,16 +19502,16 @@
       <c r="B10" s="67" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="168">
-        <v>0</v>
-      </c>
-      <c r="D10" s="168">
-        <v>0</v>
-      </c>
-      <c r="E10" s="168">
+      <c r="C10" s="19">
+        <v>0</v>
+      </c>
+      <c r="D10" s="19">
+        <v>0</v>
+      </c>
+      <c r="E10" s="19">
         <v>2000</v>
       </c>
-      <c r="F10" s="168">
+      <c r="F10" s="19">
         <v>0</v>
       </c>
       <c r="G10" s="19">
@@ -19593,7 +19538,7 @@
       <c r="N10" s="19">
         <v>0</v>
       </c>
-      <c r="O10" s="171">
+      <c r="O10" s="19">
         <v>2000</v>
       </c>
     </row>
@@ -19601,16 +19546,16 @@
       <c r="B11" s="67" t="s">
         <v>222</v>
       </c>
-      <c r="C11" s="168">
+      <c r="C11" s="19">
         <v>-19132.87</v>
       </c>
-      <c r="D11" s="168">
+      <c r="D11" s="19">
         <v>-19132.87</v>
       </c>
-      <c r="E11" s="168">
+      <c r="E11" s="19">
         <v>-18903.55</v>
       </c>
-      <c r="F11" s="168">
+      <c r="F11" s="19">
         <v>-18903.55</v>
       </c>
       <c r="G11" s="19">
@@ -19637,7 +19582,7 @@
       <c r="N11" s="19">
         <v>-19225.349999999999</v>
       </c>
-      <c r="O11" s="171">
+      <c r="O11" s="19">
         <v>-229674.75</v>
       </c>
     </row>
@@ -19645,16 +19590,16 @@
       <c r="B12" s="67" t="s">
         <v>90</v>
       </c>
-      <c r="C12" s="168">
+      <c r="C12" s="19">
         <v>3065.27</v>
       </c>
-      <c r="D12" s="168">
+      <c r="D12" s="19">
         <v>0.02</v>
       </c>
-      <c r="E12" s="168">
+      <c r="E12" s="19">
         <v>-0.14000000000000001</v>
       </c>
-      <c r="F12" s="168">
+      <c r="F12" s="19">
         <v>1024.26</v>
       </c>
       <c r="G12" s="19">
@@ -19681,7 +19626,7 @@
       <c r="N12" s="19">
         <v>0</v>
       </c>
-      <c r="O12" s="171">
+      <c r="O12" s="19">
         <v>3999.9400000000005</v>
       </c>
     </row>
@@ -19689,16 +19634,16 @@
       <c r="B13" s="67" t="s">
         <v>228</v>
       </c>
-      <c r="C13" s="168">
+      <c r="C13" s="19">
         <v>-52.82</v>
       </c>
-      <c r="D13" s="168">
-        <v>0</v>
-      </c>
-      <c r="E13" s="168">
+      <c r="D13" s="19">
+        <v>0</v>
+      </c>
+      <c r="E13" s="19">
         <v>-79.37</v>
       </c>
-      <c r="F13" s="168">
+      <c r="F13" s="19">
         <v>-24483.469999999998</v>
       </c>
       <c r="G13" s="19">
@@ -19725,7 +19670,7 @@
       <c r="N13" s="19">
         <v>-35674.22</v>
       </c>
-      <c r="O13" s="171">
+      <c r="O13" s="19">
         <v>-300408.35000000003</v>
       </c>
     </row>
@@ -19733,16 +19678,16 @@
       <c r="B14" s="67" t="s">
         <v>236</v>
       </c>
-      <c r="C14" s="168">
-        <v>0</v>
-      </c>
-      <c r="D14" s="168">
+      <c r="C14" s="19">
+        <v>0</v>
+      </c>
+      <c r="D14" s="19">
         <v>78.790000000000006</v>
       </c>
-      <c r="E14" s="168">
+      <c r="E14" s="19">
         <v>15.51</v>
       </c>
-      <c r="F14" s="168">
+      <c r="F14" s="19">
         <v>0</v>
       </c>
       <c r="G14" s="19">
@@ -19777,16 +19722,16 @@
       <c r="B15" s="67" t="s">
         <v>308</v>
       </c>
-      <c r="C15" s="168">
-        <v>0</v>
-      </c>
-      <c r="D15" s="168">
-        <v>0</v>
-      </c>
-      <c r="E15" s="168">
-        <v>0</v>
-      </c>
-      <c r="F15" s="168">
+      <c r="C15" s="19">
+        <v>0</v>
+      </c>
+      <c r="D15" s="19">
+        <v>0</v>
+      </c>
+      <c r="E15" s="19">
+        <v>0</v>
+      </c>
+      <c r="F15" s="19">
         <v>0</v>
       </c>
       <c r="G15" s="19">
@@ -19821,16 +19766,16 @@
       <c r="B16" s="67" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="168">
+      <c r="C16" s="19">
         <v>250047.3900000001</v>
       </c>
-      <c r="D16" s="168">
+      <c r="D16" s="19">
         <v>889710.84999999986</v>
       </c>
-      <c r="E16" s="168">
+      <c r="E16" s="19">
         <v>874282.35000000033</v>
       </c>
-      <c r="F16" s="168">
+      <c r="F16" s="19">
         <v>676576.85999999987</v>
       </c>
       <c r="G16" s="19">

</xml_diff>

<commit_message>
Actualizacion pedidos 23.10: comercial, MRP, tesoreria y rentabilidad
</commit_message>
<xml_diff>
--- a/Gastos/2026-Forecast-Codiagro P&L.xlsx
+++ b/Gastos/2026-Forecast-Codiagro P&L.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroquimicacodiagro365-my.sharepoint.com/personal/oscar_ocampo_codiagro_com/Documents/Escritorio/Presupuesto 2026/Calsif Comerciales/Gastos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="8_{D7C7D22D-CC9C-4A22-ADAD-C3153CF08886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86189455-F23E-4076-9388-8AB2B4892F25}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="8_{D7C7D22D-CC9C-4A22-ADAD-C3153CF08886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7764AB9F-AF8B-4975-994D-EA9D60E98D74}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="804" xr2:uid="{DA978C05-6AA7-4636-9B27-353885F16E02}"/>
+    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="804" xr2:uid="{DA978C05-6AA7-4636-9B27-353885F16E02}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="24" r:id="rId1"/>
@@ -36,9 +36,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="34" r:id="rId12"/>
-    <pivotCache cacheId="35" r:id="rId13"/>
-    <pivotCache cacheId="36" r:id="rId14"/>
+    <pivotCache cacheId="6" r:id="rId12"/>
+    <pivotCache cacheId="7" r:id="rId13"/>
+    <pivotCache cacheId="8" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1611,7 +1611,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="13">
+  <numFmts count="12">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
@@ -1624,7 +1624,6 @@
     <numFmt numFmtId="170" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="171" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="172" formatCode="#,##0.000;\(#,##0.000\);\-"/>
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="43" x14ac:knownFonts="1">
     <font>
@@ -1946,7 +1945,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="44">
+  <fills count="45">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2189,6 +2188,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2557,7 +2562,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -3096,11 +3101,14 @@
     <xf numFmtId="172" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="4" fillId="44" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="75">
     <cellStyle name="20% - Énfasis1 2" xfId="35" xr:uid="{1185DB90-4849-424E-B2AB-58A2E7F5B16C}"/>
@@ -3264,10 +3272,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9097,7 +9101,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{20404466-1C8F-4694-BEC9-2336FD9092D9}" name="TablaDinámica1" cacheId="36" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Detalle sin Ajustar">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{20404466-1C8F-4694-BEC9-2336FD9092D9}" name="TablaDinámica1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Detalle sin Ajustar">
   <location ref="B3:O16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
@@ -9392,7 +9396,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{574F8F0F-CABA-44C9-861D-B64737513C38}" name="TablaDinámica13" cacheId="35" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{574F8F0F-CABA-44C9-861D-B64737513C38}" name="TablaDinámica13" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="P3:Q12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="12">
     <pivotField numFmtId="14" showAll="0"/>
@@ -9489,7 +9493,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BCFB44B8-C86C-4350-A9CC-CF0A10A66821}" name="TablaDinámica2" cacheId="34" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BCFB44B8-C86C-4350-A9CC-CF0A10A66821}" name="TablaDinámica2" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A29:N33" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField numFmtId="14" showAll="0"/>
@@ -10203,10 +10207,10 @@
       </c>
       <c r="X6" s="77"/>
       <c r="Y6" s="78"/>
-      <c r="Z6" s="183" t="s">
+      <c r="Z6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="AA6" s="183"/>
+      <c r="AA6" s="184"/>
       <c r="AC6" s="74"/>
       <c r="AD6" s="75"/>
       <c r="AE6" s="75"/>
@@ -10215,10 +10219,10 @@
       </c>
       <c r="AG6" s="77"/>
       <c r="AH6" s="78"/>
-      <c r="AI6" s="183" t="s">
+      <c r="AI6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="AJ6" s="183"/>
+      <c r="AJ6" s="184"/>
       <c r="AL6" s="74"/>
       <c r="AM6" s="75"/>
       <c r="AN6" s="75"/>
@@ -10227,10 +10231,10 @@
       </c>
       <c r="AP6" s="77"/>
       <c r="AQ6" s="78"/>
-      <c r="AR6" s="183" t="s">
+      <c r="AR6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="AS6" s="183"/>
+      <c r="AS6" s="184"/>
       <c r="AU6" s="74"/>
       <c r="AV6" s="75"/>
       <c r="AW6" s="75"/>
@@ -10239,10 +10243,10 @@
       </c>
       <c r="AY6" s="77"/>
       <c r="AZ6" s="78"/>
-      <c r="BA6" s="183" t="s">
+      <c r="BA6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="BB6" s="183"/>
+      <c r="BB6" s="184"/>
       <c r="BD6" s="74"/>
       <c r="BE6" s="75"/>
       <c r="BF6" s="75"/>
@@ -10251,10 +10255,10 @@
       </c>
       <c r="BH6" s="77"/>
       <c r="BI6" s="78"/>
-      <c r="BJ6" s="183" t="s">
+      <c r="BJ6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="BK6" s="183"/>
+      <c r="BK6" s="184"/>
       <c r="BM6" s="74"/>
       <c r="BN6" s="75"/>
       <c r="BO6" s="75"/>
@@ -10263,10 +10267,10 @@
       </c>
       <c r="BQ6" s="77"/>
       <c r="BR6" s="78"/>
-      <c r="BS6" s="183" t="s">
+      <c r="BS6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="BT6" s="183"/>
+      <c r="BT6" s="184"/>
       <c r="BV6" s="74"/>
       <c r="BW6" s="75"/>
       <c r="BX6" s="75"/>
@@ -10275,10 +10279,10 @@
       </c>
       <c r="BZ6" s="77"/>
       <c r="CA6" s="78"/>
-      <c r="CB6" s="183" t="s">
+      <c r="CB6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="CC6" s="183"/>
+      <c r="CC6" s="184"/>
       <c r="CD6" s="103"/>
       <c r="CE6" s="74"/>
       <c r="CF6" s="75"/>
@@ -10288,10 +10292,10 @@
       </c>
       <c r="CI6" s="77"/>
       <c r="CJ6" s="78"/>
-      <c r="CK6" s="183" t="s">
+      <c r="CK6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="CL6" s="183"/>
+      <c r="CL6" s="184"/>
       <c r="CN6" s="74"/>
       <c r="CO6" s="75"/>
       <c r="CP6" s="75"/>
@@ -10300,10 +10304,10 @@
       </c>
       <c r="CR6" s="77"/>
       <c r="CS6" s="78"/>
-      <c r="CT6" s="183" t="s">
+      <c r="CT6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="CU6" s="183"/>
+      <c r="CU6" s="184"/>
       <c r="CW6" s="74"/>
       <c r="CX6" s="75"/>
       <c r="CY6" s="75"/>
@@ -10312,10 +10316,10 @@
       </c>
       <c r="DA6" s="77"/>
       <c r="DB6" s="78"/>
-      <c r="DC6" s="183" t="s">
+      <c r="DC6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="DD6" s="183"/>
+      <c r="DD6" s="184"/>
       <c r="DF6" s="74"/>
       <c r="DG6" s="75"/>
       <c r="DH6" s="75"/>
@@ -10324,16 +10328,16 @@
       </c>
       <c r="DJ6" s="77"/>
       <c r="DK6" s="78"/>
-      <c r="DL6" s="183" t="s">
+      <c r="DL6" s="184" t="s">
         <v>21</v>
       </c>
-      <c r="DM6" s="183"/>
+      <c r="DM6" s="184"/>
     </row>
     <row r="7" spans="2:117" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="80" t="s">
+      <c r="C7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="80" t="s">
@@ -10357,7 +10361,7 @@
       <c r="K7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="80" t="s">
+      <c r="L7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="M7" s="80" t="s">
@@ -10381,7 +10385,7 @@
       <c r="T7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="U7" s="80" t="s">
+      <c r="U7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="V7" s="80" t="s">
@@ -10405,7 +10409,7 @@
       <c r="AC7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="AD7" s="80" t="s">
+      <c r="AD7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="AE7" s="80" t="s">
@@ -10429,7 +10433,7 @@
       <c r="AL7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="AM7" s="80" t="s">
+      <c r="AM7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="AN7" s="80" t="s">
@@ -10453,7 +10457,7 @@
       <c r="AU7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="AV7" s="80" t="s">
+      <c r="AV7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="AW7" s="80" t="s">
@@ -10477,7 +10481,7 @@
       <c r="BD7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="BE7" s="80" t="s">
+      <c r="BE7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="BF7" s="80" t="s">
@@ -10501,7 +10505,7 @@
       <c r="BM7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="BN7" s="80" t="s">
+      <c r="BN7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="BO7" s="80" t="s">
@@ -10525,7 +10529,7 @@
       <c r="BV7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="BW7" s="80" t="s">
+      <c r="BW7" s="183" t="s">
         <v>19</v>
       </c>
       <c r="BX7" s="80" t="s">
@@ -16623,7 +16627,7 @@
       <c r="BT34" s="125">
         <v>-8.1018252585747463E-2</v>
       </c>
-      <c r="BW34" s="184">
+      <c r="BW34">
         <v>-3.6197427654381727E-2</v>
       </c>
     </row>

</xml_diff>